<commit_message>
feat: product_list.xlsx 컬럼/시트 보강 + catalog 타입 details[] 변경
[xlsx 변경]
- products 시트: detail_path 컬럼 추가 (값: 'details/1.png, 2.png, 3.png, ...')
- guide 시트 신규: 폴더 구조 + 명명 규칙 + FAQ 안내 (작업자 자급자족 매뉴얼)
- 컬럼 순서: no | product_name | folder_name | main_image | detail_path | detail_url

[catalog 타입]
- detailImage?: string → details?: string[] (배열)
- 상세 페이지 본문: details/ 폴더 안 1.png, 2.png, ... 순서대로 세로 쌓기

[효과]
- 작업자가 Excel 한 장만 봐도 어디에 어떤 파일을 만들지 명확
- 상세 이미지 갯수 제한 없음 — 1.png 부터 연속으로 추가
- 갤러리/사이즈/영상 명명은 guide 시트에서 확인

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/product_list.xlsx
+++ b/data/product_list.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet name="products" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="cats" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="guide" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -18,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="3">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -34,8 +35,27 @@
     <font>
       <color rgb="006B7280"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <color rgb="00374151"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00111827"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Consolas"/>
+      <color rgb="000F172A"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -50,6 +70,16 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="009CA3AF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="004F46E5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEF2FF"/>
       </patternFill>
     </fill>
   </fills>
@@ -79,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -91,6 +121,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -465,7 +507,7 @@
     <col width="60" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
     <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -492,7 +534,7 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>detail_image</t>
+          <t>detail_path</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -522,7 +564,7 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
@@ -552,7 +594,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
@@ -582,7 +624,7 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
@@ -612,7 +654,7 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
@@ -642,7 +684,7 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -672,7 +714,7 @@
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
@@ -702,7 +744,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
@@ -732,7 +774,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -762,7 +804,7 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -792,7 +834,7 @@
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
@@ -822,7 +864,7 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -852,7 +894,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
@@ -882,7 +924,7 @@
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
@@ -912,7 +954,7 @@
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
@@ -942,7 +984,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
@@ -972,7 +1014,7 @@
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
@@ -1002,7 +1044,7 @@
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
@@ -1032,7 +1074,7 @@
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
@@ -1062,7 +1104,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -1092,7 +1134,7 @@
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
@@ -1122,7 +1164,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
@@ -1152,7 +1194,7 @@
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
@@ -1182,7 +1224,7 @@
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
@@ -1212,7 +1254,7 @@
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
@@ -1242,7 +1284,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
@@ -1272,7 +1314,7 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
@@ -1302,7 +1344,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -1332,7 +1374,7 @@
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
@@ -1362,7 +1404,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -1392,7 +1434,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
@@ -1422,7 +1464,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -1452,7 +1494,7 @@
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
@@ -1482,7 +1524,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -1512,7 +1554,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -1542,7 +1584,7 @@
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -1572,7 +1614,7 @@
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
@@ -1602,7 +1644,7 @@
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
@@ -1632,7 +1674,7 @@
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
@@ -1662,7 +1704,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -1692,7 +1734,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
@@ -1722,7 +1764,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
@@ -1752,7 +1794,7 @@
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
@@ -1782,7 +1824,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -1812,7 +1854,7 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F45" s="2" t="inlineStr">
@@ -1842,7 +1884,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -1872,7 +1914,7 @@
       </c>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F47" s="2" t="inlineStr">
@@ -1902,7 +1944,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
@@ -1932,7 +1974,7 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
@@ -1962,7 +2004,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -1992,7 +2034,7 @@
       </c>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F51" s="2" t="inlineStr">
@@ -2022,7 +2064,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -2052,7 +2094,7 @@
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F53" s="2" t="inlineStr">
@@ -2082,7 +2124,7 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
@@ -2112,7 +2154,7 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
@@ -2142,7 +2184,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -2172,7 +2214,7 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
@@ -2202,7 +2244,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -2232,7 +2274,7 @@
       </c>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F59" s="2" t="inlineStr">
@@ -2262,7 +2304,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -2292,7 +2334,7 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F61" s="2" t="inlineStr">
@@ -2322,7 +2364,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -2352,7 +2394,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F63" s="2" t="inlineStr">
@@ -2382,7 +2424,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -2412,7 +2454,7 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F65" s="2" t="inlineStr">
@@ -2442,7 +2484,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -2472,7 +2514,7 @@
       </c>
       <c r="E67" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F67" s="2" t="inlineStr">
@@ -2502,7 +2544,7 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -2532,7 +2574,7 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
@@ -2562,7 +2604,7 @@
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -2592,7 +2634,7 @@
       </c>
       <c r="E71" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F71" s="2" t="inlineStr">
@@ -2622,7 +2664,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -2652,7 +2694,7 @@
       </c>
       <c r="E73" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F73" s="2" t="inlineStr">
@@ -2682,7 +2724,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -2712,7 +2754,7 @@
       </c>
       <c r="E75" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F75" s="2" t="inlineStr">
@@ -2742,7 +2784,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -2772,7 +2814,7 @@
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F77" s="2" t="inlineStr">
@@ -2802,7 +2844,7 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -2832,7 +2874,7 @@
       </c>
       <c r="E79" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F79" s="2" t="inlineStr">
@@ -2862,7 +2904,7 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -2892,7 +2934,7 @@
       </c>
       <c r="E81" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F81" s="2" t="inlineStr">
@@ -2922,7 +2964,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -2952,7 +2994,7 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
@@ -2982,7 +3024,7 @@
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -3012,7 +3054,7 @@
       </c>
       <c r="E85" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F85" s="2" t="inlineStr">
@@ -3042,7 +3084,7 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -3072,7 +3114,7 @@
       </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F87" s="2" t="inlineStr">
@@ -3102,7 +3144,7 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
@@ -3132,7 +3174,7 @@
       </c>
       <c r="E89" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F89" s="2" t="inlineStr">
@@ -3162,7 +3204,7 @@
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
@@ -3192,7 +3234,7 @@
       </c>
       <c r="E91" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F91" s="2" t="inlineStr">
@@ -3222,7 +3264,7 @@
       </c>
       <c r="E92" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F92" s="2" t="inlineStr">
@@ -3252,7 +3294,7 @@
       </c>
       <c r="E93" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F93" s="2" t="inlineStr">
@@ -3282,7 +3324,7 @@
       </c>
       <c r="E94" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F94" s="2" t="inlineStr">
@@ -3312,7 +3354,7 @@
       </c>
       <c r="E95" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F95" s="2" t="inlineStr">
@@ -3342,7 +3384,7 @@
       </c>
       <c r="E96" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F96" s="2" t="inlineStr">
@@ -3372,7 +3414,7 @@
       </c>
       <c r="E97" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F97" s="2" t="inlineStr">
@@ -3402,7 +3444,7 @@
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F98" s="2" t="inlineStr">
@@ -3432,7 +3474,7 @@
       </c>
       <c r="E99" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F99" s="2" t="inlineStr">
@@ -3462,7 +3504,7 @@
       </c>
       <c r="E100" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F100" s="2" t="inlineStr">
@@ -3492,7 +3534,7 @@
       </c>
       <c r="E101" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F101" s="2" t="inlineStr">
@@ -3522,7 +3564,7 @@
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
@@ -3552,7 +3594,7 @@
       </c>
       <c r="E103" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F103" s="2" t="inlineStr">
@@ -3582,7 +3624,7 @@
       </c>
       <c r="E104" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F104" s="2" t="inlineStr">
@@ -3612,7 +3654,7 @@
       </c>
       <c r="E105" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F105" s="2" t="inlineStr">
@@ -3642,7 +3684,7 @@
       </c>
       <c r="E106" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F106" s="2" t="inlineStr">
@@ -3672,7 +3714,7 @@
       </c>
       <c r="E107" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F107" s="2" t="inlineStr">
@@ -3702,7 +3744,7 @@
       </c>
       <c r="E108" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F108" s="2" t="inlineStr">
@@ -3732,7 +3774,7 @@
       </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F109" s="2" t="inlineStr">
@@ -3762,7 +3804,7 @@
       </c>
       <c r="E110" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F110" s="2" t="inlineStr">
@@ -3792,7 +3834,7 @@
       </c>
       <c r="E111" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F111" s="2" t="inlineStr">
@@ -3822,7 +3864,7 @@
       </c>
       <c r="E112" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F112" s="2" t="inlineStr">
@@ -3852,7 +3894,7 @@
       </c>
       <c r="E113" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F113" s="2" t="inlineStr">
@@ -3882,7 +3924,7 @@
       </c>
       <c r="E114" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F114" s="2" t="inlineStr">
@@ -3912,7 +3954,7 @@
       </c>
       <c r="E115" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F115" s="2" t="inlineStr">
@@ -3942,7 +3984,7 @@
       </c>
       <c r="E116" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F116" s="2" t="inlineStr">
@@ -3972,7 +4014,7 @@
       </c>
       <c r="E117" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F117" s="2" t="inlineStr">
@@ -4002,7 +4044,7 @@
       </c>
       <c r="E118" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F118" s="2" t="inlineStr">
@@ -4032,7 +4074,7 @@
       </c>
       <c r="E119" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F119" s="2" t="inlineStr">
@@ -4062,7 +4104,7 @@
       </c>
       <c r="E120" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F120" s="2" t="inlineStr">
@@ -4092,7 +4134,7 @@
       </c>
       <c r="E121" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F121" s="2" t="inlineStr">
@@ -4122,7 +4164,7 @@
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F122" s="2" t="inlineStr">
@@ -4152,7 +4194,7 @@
       </c>
       <c r="E123" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F123" s="2" t="inlineStr">
@@ -4182,7 +4224,7 @@
       </c>
       <c r="E124" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F124" s="2" t="inlineStr">
@@ -4212,7 +4254,7 @@
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F125" s="2" t="inlineStr">
@@ -4242,7 +4284,7 @@
       </c>
       <c r="E126" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F126" s="2" t="inlineStr">
@@ -4272,7 +4314,7 @@
       </c>
       <c r="E127" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F127" s="2" t="inlineStr">
@@ -4302,7 +4344,7 @@
       </c>
       <c r="E128" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F128" s="2" t="inlineStr">
@@ -4332,7 +4374,7 @@
       </c>
       <c r="E129" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F129" s="2" t="inlineStr">
@@ -4362,7 +4404,7 @@
       </c>
       <c r="E130" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F130" s="2" t="inlineStr">
@@ -4392,7 +4434,7 @@
       </c>
       <c r="E131" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F131" s="2" t="inlineStr">
@@ -4422,7 +4464,7 @@
       </c>
       <c r="E132" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F132" s="2" t="inlineStr">
@@ -4452,7 +4494,7 @@
       </c>
       <c r="E133" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F133" s="2" t="inlineStr">
@@ -4482,7 +4524,7 @@
       </c>
       <c r="E134" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F134" s="2" t="inlineStr">
@@ -4512,7 +4554,7 @@
       </c>
       <c r="E135" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F135" s="2" t="inlineStr">
@@ -4542,7 +4584,7 @@
       </c>
       <c r="E136" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F136" s="2" t="inlineStr">
@@ -4572,7 +4614,7 @@
       </c>
       <c r="E137" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F137" s="2" t="inlineStr">
@@ -4602,7 +4644,7 @@
       </c>
       <c r="E138" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F138" s="2" t="inlineStr">
@@ -4632,7 +4674,7 @@
       </c>
       <c r="E139" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F139" s="2" t="inlineStr">
@@ -4662,7 +4704,7 @@
       </c>
       <c r="E140" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F140" s="2" t="inlineStr">
@@ -4692,7 +4734,7 @@
       </c>
       <c r="E141" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F141" s="2" t="inlineStr">
@@ -4722,7 +4764,7 @@
       </c>
       <c r="E142" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F142" s="2" t="inlineStr">
@@ -4752,7 +4794,7 @@
       </c>
       <c r="E143" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F143" s="2" t="inlineStr">
@@ -4782,7 +4824,7 @@
       </c>
       <c r="E144" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F144" s="2" t="inlineStr">
@@ -4812,7 +4854,7 @@
       </c>
       <c r="E145" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F145" s="2" t="inlineStr">
@@ -4842,7 +4884,7 @@
       </c>
       <c r="E146" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F146" s="2" t="inlineStr">
@@ -4872,7 +4914,7 @@
       </c>
       <c r="E147" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F147" s="2" t="inlineStr">
@@ -4902,7 +4944,7 @@
       </c>
       <c r="E148" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F148" s="2" t="inlineStr">
@@ -4932,7 +4974,7 @@
       </c>
       <c r="E149" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F149" s="2" t="inlineStr">
@@ -4962,7 +5004,7 @@
       </c>
       <c r="E150" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F150" s="2" t="inlineStr">
@@ -4992,7 +5034,7 @@
       </c>
       <c r="E151" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F151" s="2" t="inlineStr">
@@ -5022,7 +5064,7 @@
       </c>
       <c r="E152" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F152" s="2" t="inlineStr">
@@ -5052,7 +5094,7 @@
       </c>
       <c r="E153" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F153" s="2" t="inlineStr">
@@ -5082,7 +5124,7 @@
       </c>
       <c r="E154" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F154" s="2" t="inlineStr">
@@ -5112,7 +5154,7 @@
       </c>
       <c r="E155" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F155" s="2" t="inlineStr">
@@ -5142,7 +5184,7 @@
       </c>
       <c r="E156" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F156" s="2" t="inlineStr">
@@ -5172,7 +5214,7 @@
       </c>
       <c r="E157" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F157" s="2" t="inlineStr">
@@ -5202,7 +5244,7 @@
       </c>
       <c r="E158" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F158" s="2" t="inlineStr">
@@ -5232,7 +5274,7 @@
       </c>
       <c r="E159" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F159" s="2" t="inlineStr">
@@ -5262,7 +5304,7 @@
       </c>
       <c r="E160" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F160" s="2" t="inlineStr">
@@ -5292,7 +5334,7 @@
       </c>
       <c r="E161" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F161" s="2" t="inlineStr">
@@ -5322,7 +5364,7 @@
       </c>
       <c r="E162" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F162" s="2" t="inlineStr">
@@ -5352,7 +5394,7 @@
       </c>
       <c r="E163" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F163" s="2" t="inlineStr">
@@ -5382,7 +5424,7 @@
       </c>
       <c r="E164" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F164" s="2" t="inlineStr">
@@ -5412,7 +5454,7 @@
       </c>
       <c r="E165" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F165" s="2" t="inlineStr">
@@ -5442,7 +5484,7 @@
       </c>
       <c r="E166" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F166" s="2" t="inlineStr">
@@ -5472,7 +5514,7 @@
       </c>
       <c r="E167" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F167" s="2" t="inlineStr">
@@ -5502,7 +5544,7 @@
       </c>
       <c r="E168" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F168" s="2" t="inlineStr">
@@ -5532,7 +5574,7 @@
       </c>
       <c r="E169" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F169" s="2" t="inlineStr">
@@ -5562,7 +5604,7 @@
       </c>
       <c r="E170" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F170" s="2" t="inlineStr">
@@ -5592,7 +5634,7 @@
       </c>
       <c r="E171" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F171" s="2" t="inlineStr">
@@ -5622,7 +5664,7 @@
       </c>
       <c r="E172" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F172" s="2" t="inlineStr">
@@ -5652,7 +5694,7 @@
       </c>
       <c r="E173" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F173" s="2" t="inlineStr">
@@ -5682,7 +5724,7 @@
       </c>
       <c r="E174" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F174" s="2" t="inlineStr">
@@ -5712,7 +5754,7 @@
       </c>
       <c r="E175" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F175" s="2" t="inlineStr">
@@ -5742,7 +5784,7 @@
       </c>
       <c r="E176" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F176" s="2" t="inlineStr">
@@ -5772,7 +5814,7 @@
       </c>
       <c r="E177" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F177" s="2" t="inlineStr">
@@ -5802,7 +5844,7 @@
       </c>
       <c r="E178" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F178" s="2" t="inlineStr">
@@ -5832,7 +5874,7 @@
       </c>
       <c r="E179" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F179" s="2" t="inlineStr">
@@ -5862,7 +5904,7 @@
       </c>
       <c r="E180" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F180" s="2" t="inlineStr">
@@ -5892,7 +5934,7 @@
       </c>
       <c r="E181" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F181" s="2" t="inlineStr">
@@ -5922,7 +5964,7 @@
       </c>
       <c r="E182" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F182" s="2" t="inlineStr">
@@ -5952,7 +5994,7 @@
       </c>
       <c r="E183" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F183" s="2" t="inlineStr">
@@ -5982,7 +6024,7 @@
       </c>
       <c r="E184" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F184" s="2" t="inlineStr">
@@ -6012,7 +6054,7 @@
       </c>
       <c r="E185" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F185" s="2" t="inlineStr">
@@ -6042,7 +6084,7 @@
       </c>
       <c r="E186" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F186" s="2" t="inlineStr">
@@ -6072,7 +6114,7 @@
       </c>
       <c r="E187" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F187" s="2" t="inlineStr">
@@ -6102,7 +6144,7 @@
       </c>
       <c r="E188" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F188" s="2" t="inlineStr">
@@ -6132,7 +6174,7 @@
       </c>
       <c r="E189" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F189" s="2" t="inlineStr">
@@ -6162,7 +6204,7 @@
       </c>
       <c r="E190" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F190" s="2" t="inlineStr">
@@ -6192,7 +6234,7 @@
       </c>
       <c r="E191" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F191" s="2" t="inlineStr">
@@ -6222,7 +6264,7 @@
       </c>
       <c r="E192" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F192" s="2" t="inlineStr">
@@ -6252,7 +6294,7 @@
       </c>
       <c r="E193" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F193" s="2" t="inlineStr">
@@ -6282,7 +6324,7 @@
       </c>
       <c r="E194" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F194" s="2" t="inlineStr">
@@ -6312,7 +6354,7 @@
       </c>
       <c r="E195" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F195" s="2" t="inlineStr">
@@ -6342,7 +6384,7 @@
       </c>
       <c r="E196" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F196" s="2" t="inlineStr">
@@ -6372,7 +6414,7 @@
       </c>
       <c r="E197" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F197" s="2" t="inlineStr">
@@ -6402,7 +6444,7 @@
       </c>
       <c r="E198" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F198" s="2" t="inlineStr">
@@ -6432,7 +6474,7 @@
       </c>
       <c r="E199" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F199" s="2" t="inlineStr">
@@ -6462,7 +6504,7 @@
       </c>
       <c r="E200" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F200" s="2" t="inlineStr">
@@ -6492,7 +6534,7 @@
       </c>
       <c r="E201" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F201" s="2" t="inlineStr">
@@ -6522,7 +6564,7 @@
       </c>
       <c r="E202" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F202" s="2" t="inlineStr">
@@ -6552,7 +6594,7 @@
       </c>
       <c r="E203" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F203" s="2" t="inlineStr">
@@ -6582,7 +6624,7 @@
       </c>
       <c r="E204" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F204" s="2" t="inlineStr">
@@ -6612,7 +6654,7 @@
       </c>
       <c r="E205" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F205" s="2" t="inlineStr">
@@ -6642,7 +6684,7 @@
       </c>
       <c r="E206" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F206" s="2" t="inlineStr">
@@ -6672,7 +6714,7 @@
       </c>
       <c r="E207" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F207" s="2" t="inlineStr">
@@ -6702,7 +6744,7 @@
       </c>
       <c r="E208" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F208" s="2" t="inlineStr">
@@ -6732,7 +6774,7 @@
       </c>
       <c r="E209" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F209" s="2" t="inlineStr">
@@ -6762,7 +6804,7 @@
       </c>
       <c r="E210" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F210" s="2" t="inlineStr">
@@ -6792,7 +6834,7 @@
       </c>
       <c r="E211" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F211" s="2" t="inlineStr">
@@ -6822,7 +6864,7 @@
       </c>
       <c r="E212" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F212" s="2" t="inlineStr">
@@ -6852,7 +6894,7 @@
       </c>
       <c r="E213" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F213" s="2" t="inlineStr">
@@ -6882,7 +6924,7 @@
       </c>
       <c r="E214" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F214" s="2" t="inlineStr">
@@ -6912,7 +6954,7 @@
       </c>
       <c r="E215" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F215" s="2" t="inlineStr">
@@ -6942,7 +6984,7 @@
       </c>
       <c r="E216" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F216" s="2" t="inlineStr">
@@ -6972,7 +7014,7 @@
       </c>
       <c r="E217" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F217" s="2" t="inlineStr">
@@ -7002,7 +7044,7 @@
       </c>
       <c r="E218" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F218" s="2" t="inlineStr">
@@ -7032,7 +7074,7 @@
       </c>
       <c r="E219" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F219" s="2" t="inlineStr">
@@ -7062,7 +7104,7 @@
       </c>
       <c r="E220" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F220" s="2" t="inlineStr">
@@ -7092,7 +7134,7 @@
       </c>
       <c r="E221" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F221" s="2" t="inlineStr">
@@ -7122,7 +7164,7 @@
       </c>
       <c r="E222" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F222" s="2" t="inlineStr">
@@ -7152,7 +7194,7 @@
       </c>
       <c r="E223" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F223" s="2" t="inlineStr">
@@ -7182,7 +7224,7 @@
       </c>
       <c r="E224" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F224" s="2" t="inlineStr">
@@ -7212,7 +7254,7 @@
       </c>
       <c r="E225" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F225" s="2" t="inlineStr">
@@ -7242,7 +7284,7 @@
       </c>
       <c r="E226" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F226" s="2" t="inlineStr">
@@ -7272,7 +7314,7 @@
       </c>
       <c r="E227" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F227" s="2" t="inlineStr">
@@ -7302,7 +7344,7 @@
       </c>
       <c r="E228" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F228" s="2" t="inlineStr">
@@ -7332,7 +7374,7 @@
       </c>
       <c r="E229" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F229" s="2" t="inlineStr">
@@ -7362,7 +7404,7 @@
       </c>
       <c r="E230" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F230" s="2" t="inlineStr">
@@ -7392,7 +7434,7 @@
       </c>
       <c r="E231" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F231" s="2" t="inlineStr">
@@ -7422,7 +7464,7 @@
       </c>
       <c r="E232" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F232" s="2" t="inlineStr">
@@ -7452,7 +7494,7 @@
       </c>
       <c r="E233" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F233" s="2" t="inlineStr">
@@ -7482,7 +7524,7 @@
       </c>
       <c r="E234" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F234" s="2" t="inlineStr">
@@ -7512,7 +7554,7 @@
       </c>
       <c r="E235" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F235" s="2" t="inlineStr">
@@ -7542,7 +7584,7 @@
       </c>
       <c r="E236" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F236" s="2" t="inlineStr">
@@ -7572,7 +7614,7 @@
       </c>
       <c r="E237" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F237" s="2" t="inlineStr">
@@ -7602,7 +7644,7 @@
       </c>
       <c r="E238" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F238" s="2" t="inlineStr">
@@ -7632,7 +7674,7 @@
       </c>
       <c r="E239" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F239" s="2" t="inlineStr">
@@ -7662,7 +7704,7 @@
       </c>
       <c r="E240" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F240" s="2" t="inlineStr">
@@ -7692,7 +7734,7 @@
       </c>
       <c r="E241" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F241" s="2" t="inlineStr">
@@ -7722,7 +7764,7 @@
       </c>
       <c r="E242" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F242" s="2" t="inlineStr">
@@ -7752,7 +7794,7 @@
       </c>
       <c r="E243" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F243" s="2" t="inlineStr">
@@ -7782,7 +7824,7 @@
       </c>
       <c r="E244" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F244" s="2" t="inlineStr">
@@ -7812,7 +7854,7 @@
       </c>
       <c r="E245" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F245" s="2" t="inlineStr">
@@ -7842,7 +7884,7 @@
       </c>
       <c r="E246" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F246" s="2" t="inlineStr">
@@ -7872,7 +7914,7 @@
       </c>
       <c r="E247" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F247" s="2" t="inlineStr">
@@ -7902,7 +7944,7 @@
       </c>
       <c r="E248" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F248" s="2" t="inlineStr">
@@ -7932,7 +7974,7 @@
       </c>
       <c r="E249" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F249" s="2" t="inlineStr">
@@ -7962,7 +8004,7 @@
       </c>
       <c r="E250" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F250" s="2" t="inlineStr">
@@ -7992,7 +8034,7 @@
       </c>
       <c r="E251" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F251" s="2" t="inlineStr">
@@ -8022,7 +8064,7 @@
       </c>
       <c r="E252" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F252" s="2" t="inlineStr">
@@ -8052,7 +8094,7 @@
       </c>
       <c r="E253" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F253" s="2" t="inlineStr">
@@ -8082,7 +8124,7 @@
       </c>
       <c r="E254" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F254" s="2" t="inlineStr">
@@ -8112,7 +8154,7 @@
       </c>
       <c r="E255" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F255" s="2" t="inlineStr">
@@ -8142,7 +8184,7 @@
       </c>
       <c r="E256" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F256" s="2" t="inlineStr">
@@ -8172,7 +8214,7 @@
       </c>
       <c r="E257" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F257" s="2" t="inlineStr">
@@ -8202,7 +8244,7 @@
       </c>
       <c r="E258" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F258" s="2" t="inlineStr">
@@ -8232,7 +8274,7 @@
       </c>
       <c r="E259" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F259" s="2" t="inlineStr">
@@ -8262,7 +8304,7 @@
       </c>
       <c r="E260" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F260" s="2" t="inlineStr">
@@ -8292,7 +8334,7 @@
       </c>
       <c r="E261" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F261" s="2" t="inlineStr">
@@ -8322,7 +8364,7 @@
       </c>
       <c r="E262" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F262" s="2" t="inlineStr">
@@ -8352,7 +8394,7 @@
       </c>
       <c r="E263" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F263" s="2" t="inlineStr">
@@ -8382,7 +8424,7 @@
       </c>
       <c r="E264" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F264" s="2" t="inlineStr">
@@ -8412,7 +8454,7 @@
       </c>
       <c r="E265" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F265" s="2" t="inlineStr">
@@ -8442,7 +8484,7 @@
       </c>
       <c r="E266" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F266" s="2" t="inlineStr">
@@ -8472,7 +8514,7 @@
       </c>
       <c r="E267" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F267" s="2" t="inlineStr">
@@ -8502,7 +8544,7 @@
       </c>
       <c r="E268" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F268" s="2" t="inlineStr">
@@ -8532,7 +8574,7 @@
       </c>
       <c r="E269" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F269" s="2" t="inlineStr">
@@ -8562,7 +8604,7 @@
       </c>
       <c r="E270" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F270" s="2" t="inlineStr">
@@ -8592,7 +8634,7 @@
       </c>
       <c r="E271" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F271" s="2" t="inlineStr">
@@ -8622,7 +8664,7 @@
       </c>
       <c r="E272" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F272" s="2" t="inlineStr">
@@ -8652,7 +8694,7 @@
       </c>
       <c r="E273" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F273" s="2" t="inlineStr">
@@ -8682,7 +8724,7 @@
       </c>
       <c r="E274" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F274" s="2" t="inlineStr">
@@ -8712,7 +8754,7 @@
       </c>
       <c r="E275" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F275" s="2" t="inlineStr">
@@ -8742,7 +8784,7 @@
       </c>
       <c r="E276" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F276" s="2" t="inlineStr">
@@ -8772,7 +8814,7 @@
       </c>
       <c r="E277" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F277" s="2" t="inlineStr">
@@ -8802,7 +8844,7 @@
       </c>
       <c r="E278" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F278" s="2" t="inlineStr">
@@ -8832,7 +8874,7 @@
       </c>
       <c r="E279" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F279" s="2" t="inlineStr">
@@ -8862,7 +8904,7 @@
       </c>
       <c r="E280" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F280" s="2" t="inlineStr">
@@ -8892,7 +8934,7 @@
       </c>
       <c r="E281" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F281" s="2" t="inlineStr">
@@ -8922,7 +8964,7 @@
       </c>
       <c r="E282" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F282" s="2" t="inlineStr">
@@ -8952,7 +8994,7 @@
       </c>
       <c r="E283" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F283" s="2" t="inlineStr">
@@ -8982,7 +9024,7 @@
       </c>
       <c r="E284" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F284" s="2" t="inlineStr">
@@ -9012,7 +9054,7 @@
       </c>
       <c r="E285" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F285" s="2" t="inlineStr">
@@ -9042,7 +9084,7 @@
       </c>
       <c r="E286" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F286" s="2" t="inlineStr">
@@ -9072,7 +9114,7 @@
       </c>
       <c r="E287" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F287" s="2" t="inlineStr">
@@ -9102,7 +9144,7 @@
       </c>
       <c r="E288" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F288" s="2" t="inlineStr">
@@ -9132,7 +9174,7 @@
       </c>
       <c r="E289" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F289" s="2" t="inlineStr">
@@ -9162,7 +9204,7 @@
       </c>
       <c r="E290" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F290" s="2" t="inlineStr">
@@ -9192,7 +9234,7 @@
       </c>
       <c r="E291" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F291" s="2" t="inlineStr">
@@ -9222,7 +9264,7 @@
       </c>
       <c r="E292" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F292" s="2" t="inlineStr">
@@ -9252,7 +9294,7 @@
       </c>
       <c r="E293" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F293" s="2" t="inlineStr">
@@ -9282,7 +9324,7 @@
       </c>
       <c r="E294" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F294" s="2" t="inlineStr">
@@ -9312,7 +9354,7 @@
       </c>
       <c r="E295" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F295" s="2" t="inlineStr">
@@ -9342,7 +9384,7 @@
       </c>
       <c r="E296" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F296" s="2" t="inlineStr">
@@ -9372,7 +9414,7 @@
       </c>
       <c r="E297" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F297" s="2" t="inlineStr">
@@ -9402,7 +9444,7 @@
       </c>
       <c r="E298" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F298" s="2" t="inlineStr">
@@ -9432,7 +9474,7 @@
       </c>
       <c r="E299" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F299" s="2" t="inlineStr">
@@ -9462,7 +9504,7 @@
       </c>
       <c r="E300" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F300" s="2" t="inlineStr">
@@ -9492,7 +9534,7 @@
       </c>
       <c r="E301" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F301" s="2" t="inlineStr">
@@ -9522,7 +9564,7 @@
       </c>
       <c r="E302" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F302" s="2" t="inlineStr">
@@ -9552,7 +9594,7 @@
       </c>
       <c r="E303" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F303" s="2" t="inlineStr">
@@ -9582,7 +9624,7 @@
       </c>
       <c r="E304" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F304" s="2" t="inlineStr">
@@ -9612,7 +9654,7 @@
       </c>
       <c r="E305" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F305" s="2" t="inlineStr">
@@ -9642,7 +9684,7 @@
       </c>
       <c r="E306" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F306" s="2" t="inlineStr">
@@ -9672,7 +9714,7 @@
       </c>
       <c r="E307" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F307" s="2" t="inlineStr">
@@ -9702,7 +9744,7 @@
       </c>
       <c r="E308" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F308" s="2" t="inlineStr">
@@ -9732,7 +9774,7 @@
       </c>
       <c r="E309" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F309" s="2" t="inlineStr">
@@ -9762,7 +9804,7 @@
       </c>
       <c r="E310" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F310" s="2" t="inlineStr">
@@ -9792,7 +9834,7 @@
       </c>
       <c r="E311" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F311" s="2" t="inlineStr">
@@ -9822,7 +9864,7 @@
       </c>
       <c r="E312" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F312" s="2" t="inlineStr">
@@ -9852,7 +9894,7 @@
       </c>
       <c r="E313" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F313" s="2" t="inlineStr">
@@ -9882,7 +9924,7 @@
       </c>
       <c r="E314" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F314" s="2" t="inlineStr">
@@ -9912,7 +9954,7 @@
       </c>
       <c r="E315" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F315" s="2" t="inlineStr">
@@ -9942,7 +9984,7 @@
       </c>
       <c r="E316" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F316" s="2" t="inlineStr">
@@ -9972,7 +10014,7 @@
       </c>
       <c r="E317" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F317" s="2" t="inlineStr">
@@ -10002,7 +10044,7 @@
       </c>
       <c r="E318" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F318" s="2" t="inlineStr">
@@ -10032,7 +10074,7 @@
       </c>
       <c r="E319" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F319" s="2" t="inlineStr">
@@ -10062,7 +10104,7 @@
       </c>
       <c r="E320" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F320" s="2" t="inlineStr">
@@ -10092,7 +10134,7 @@
       </c>
       <c r="E321" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F321" s="2" t="inlineStr">
@@ -10122,7 +10164,7 @@
       </c>
       <c r="E322" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F322" s="2" t="inlineStr">
@@ -10152,7 +10194,7 @@
       </c>
       <c r="E323" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F323" s="2" t="inlineStr">
@@ -10182,7 +10224,7 @@
       </c>
       <c r="E324" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F324" s="2" t="inlineStr">
@@ -10212,7 +10254,7 @@
       </c>
       <c r="E325" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F325" s="2" t="inlineStr">
@@ -10242,7 +10284,7 @@
       </c>
       <c r="E326" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F326" s="2" t="inlineStr">
@@ -10272,7 +10314,7 @@
       </c>
       <c r="E327" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F327" s="2" t="inlineStr">
@@ -10302,7 +10344,7 @@
       </c>
       <c r="E328" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F328" s="2" t="inlineStr">
@@ -10332,7 +10374,7 @@
       </c>
       <c r="E329" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F329" s="2" t="inlineStr">
@@ -10362,7 +10404,7 @@
       </c>
       <c r="E330" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F330" s="2" t="inlineStr">
@@ -10392,7 +10434,7 @@
       </c>
       <c r="E331" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F331" s="2" t="inlineStr">
@@ -10422,7 +10464,7 @@
       </c>
       <c r="E332" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F332" s="2" t="inlineStr">
@@ -10452,7 +10494,7 @@
       </c>
       <c r="E333" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F333" s="2" t="inlineStr">
@@ -10482,7 +10524,7 @@
       </c>
       <c r="E334" s="2" t="inlineStr">
         <is>
-          <t>info.png</t>
+          <t>details/1.png, 2.png, 3.png, ...</t>
         </is>
       </c>
       <c r="F334" s="2" t="inlineStr">
@@ -10794,4 +10836,327 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E50"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="120" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="5" t="inlineStr">
+        <is>
+          <t>product_list.xlsx 작업 가이드</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="6" t="inlineStr"/>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>● 작업 위치</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="6" t="inlineStr"/>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  각 제품의 자산은 D:/Daengdabang/products/{folder_name}/ 폴더에 보관합니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  folder_name 은 products 시트의 folder_name 컬럼에서 확인.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="A7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>● 폴더 구조 (예시: rw_notarock)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="6" t="inlineStr"/>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  D:/Daengdabang/products/rw_notarock/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ├── rw_notarock.png    ← 메인 이미지 (필수, folder_name + .png)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ├── 2.png              ← 갤러리 2번째 (옵션, 정사각형 권장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ├── 3.png              ← 갤러리 3번째</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ├── 4.png, 5.png, ...  ← 추가 갤러리 (필요한 만큼)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ├── size.png           ← 사이즈 차트 (옵션)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  ├── video.mp4          ← 영상 (옵션, mp4 + h.264)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  └── details/           ← 상세 페이지 본문 (긴 세로 이미지들)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      ├── 1.png          ← 상세 1번째 (헤더/배너)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      ├── 2.png          ← 상세 2번째 (제품 소개)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      ├── 3.png          ← 상세 3번째 (특징)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      └── ...            ← 필요한 만큼 (사이트가 1.png 부터 순서대로 표시)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="6" t="inlineStr"/>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
+        <is>
+          <t>● 파일 명명 규칙</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="6" t="inlineStr"/>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  메인 이미지: folder_name 과 동일 + .png</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">              예) folder_name = 'rw_notarock' → rw_notarock.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  갤러리:     2.png 부터 시작 (메인이 1번째이므로)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  상세 본문:  details/ 폴더 안에 1.png 부터 순서대로</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  사이즈:     size.png (고정 파일명)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="18" customHeight="1">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  영상:       video.mp4 (고정 파일명, mp4 권장)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="6" t="inlineStr"/>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="7" t="inlineStr">
+        <is>
+          <t>● 업로드 후 사이트 반영</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="6" t="inlineStr"/>
+    </row>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1. 파일을 위 폴더에 저장</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2. GitHub 에 push (또는 RPA 자동)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="18" customHeight="1">
+      <c r="A36" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  3. 1~2분 후 detail_url 에서 확인</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="6" t="inlineStr"/>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="7" t="inlineStr">
+        <is>
+          <t>● 자주 묻는 질문</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="18" customHeight="1">
+      <c r="A39" s="6" t="inlineStr"/>
+    </row>
+    <row r="40" ht="18" customHeight="1">
+      <c r="A40" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Q. 폴더 안에 파일을 넣었는데 사이트에 안 보입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="18" customHeight="1">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A. 1~2분 정도 빌드/배포 시간 필요. 그래도 안 보이면 파일명 확인 (오타·확장자).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="18" customHeight="1">
+      <c r="A42" s="6" t="inlineStr"/>
+    </row>
+    <row r="43" ht="18" customHeight="1">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Q. 갤러리 사진 갯수에 제한이 있나요?</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A. 제한 없음. 2.png 부터 빈 번호 없이 연속으로 추가.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="6" t="inlineStr"/>
+    </row>
+    <row r="46" ht="18" customHeight="1">
+      <c r="A46" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Q. 상세 이미지 1번 위에 헤더, 마지막에 푸터 같은 게 있어야 하나요?</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="18" customHeight="1">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A. 자유. 사이트는 1.png 부터 순서대로만 보여줍니다. 디자인은 자유.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="6" t="inlineStr"/>
+    </row>
+    <row r="49" ht="18" customHeight="1">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Q. 모든 제품에 영상이나 사이즈 차트가 필요한가요?</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="18" customHeight="1">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A. 아니요. 있으면 표시, 없으면 그 영역 자체가 안 보임. 옵션입니다.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A32:E32"/>
+    <mergeCell ref="A8:E8"/>
+    <mergeCell ref="A3:E3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: sync-images.mjs (자동 카탈로그 동기화) + predev/prebuild 훅
[sync-images.mjs]
- public/images/products/catalog/{folder}/ 폴더 스캔
- 자동 감지 후 catalog.json 갱신:
  - {folder}.png → image
  - 2.png, 3.png, ... → gallery[]
  - details/1.png, 2.png, ... → details[]
  - size.png → sizeImage
  - video.mp4 → video (로컬 파일 우선, 없으면 외부 URL 보존)
- 변경 없으면 catalog.json 안 건드림 (incremental)
- 333개 폴더 처리에 약 0.7초

[package.json]
- npm run sync-images (수동 실행)
- predev: npm run dev 직전 자동 실행
- prebuild: npm run build 직전 자동 실행
- → 작업자는 폴더에 파일만 두면 끝, 별도 명령 불필요

[product_list.xlsx guide 시트]
- 작업 위치 안내 갱신:
  D:/Daengdabang/products/ (개인 PC) → public/images/products/catalog/ (git 공유)
- 협업 친화 — git clone 하면 모든 자산 따라옴
- 자주 묻는 질문 보강 (sync-images 동작 설명 등)

[효과]
- 외부 폴더 D:/Daengdabang/products/ 불필요 (수동 삭제 가능)
- 단일 출처 — public/ 이 진실
- 모든 협업자가 git clone 한 번으로 동일 환경
- 작업 흐름: 파일 추가 → npm run dev → commit/push → 끝

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/product_list.xlsx
+++ b/data/product_list.xlsx
@@ -10844,7 +10844,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -10863,7 +10863,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>● 작업 위치</t>
+          <t>● 작업 위치 (모든 협업자 공통)</t>
         </is>
       </c>
     </row>
@@ -10873,14 +10873,14 @@
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  각 제품의 자산은 D:/Daengdabang/products/{folder_name}/ 폴더에 보관합니다.</t>
+          <t xml:space="preserve">  각 제품의 자산은 git 저장소 안의 아래 폴더에 보관합니다:</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  folder_name 은 products 시트의 folder_name 컬럼에서 확인.</t>
+          <t xml:space="preserve">  Daengdabang_Shop/public/images/products/catalog/{folder_name}/</t>
         </is>
       </c>
     </row>
@@ -10888,212 +10888,216 @@
       <c r="A7" s="6" t="inlineStr"/>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  folder_name 은 products 시트의 folder_name 컬럼에서 확인.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  git clone 으로 받으면 모든 자산이 함께 따라옵니다 — 별도 폴더 공유 불필요.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="6" t="inlineStr"/>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>● 폴더 구조 (예시: rw_notarock)</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="6" t="inlineStr"/>
-    </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  D:/Daengdabang/products/rw_notarock/</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ├── rw_notarock.png    ← 메인 이미지 (필수, folder_name + .png)</t>
-        </is>
-      </c>
-    </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ├── 2.png              ← 갤러리 2번째 (옵션, 정사각형 권장)</t>
-        </is>
-      </c>
+      <c r="A12" s="6" t="inlineStr"/>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  ├── 3.png              ← 갤러리 3번째</t>
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Daengdabang_Shop/public/images/products/catalog/rw_notarock/</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ├── 4.png, 5.png, ...  ← 추가 갤러리 (필요한 만큼)</t>
+          <t xml:space="preserve">  ├── rw_notarock.png    ← 메인 이미지 (필수, folder_name + .png)</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ├── size.png           ← 사이즈 차트 (옵션)</t>
+          <t xml:space="preserve">  ├── 2.png              ← 갤러리 2번째 (옵션, 정사각형 권장)</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ├── video.mp4          ← 영상 (옵션, mp4 + h.264)</t>
+          <t xml:space="preserve">  ├── 3.png              ← 갤러리 3번째</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">  └── details/           ← 상세 페이지 본문 (긴 세로 이미지들)</t>
+          <t xml:space="preserve">  ├── 4.png, 5.png, ...  ← 추가 갤러리 (필요한 만큼)</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">      ├── 1.png          ← 상세 1번째 (헤더/배너)</t>
+          <t xml:space="preserve">  ├── size.png           ← 사이즈 차트 (옵션)</t>
         </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">      ├── 2.png          ← 상세 2번째 (제품 소개)</t>
+          <t xml:space="preserve">  ├── video.mp4          ← 영상 (옵션, mp4 + h.264)</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">      ├── 3.png          ← 상세 3번째 (특징)</t>
+          <t xml:space="preserve">  └── details/           ← 상세 페이지 본문 (긴 세로 이미지들)</t>
         </is>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">      ├── 1.png          ← 상세 1번째 (헤더/배너)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      ├── 2.png          ← 상세 2번째 (제품 소개)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">      ├── 3.png          ← 상세 3번째 (특징)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">      └── ...            ← 필요한 만큼 (사이트가 1.png 부터 순서대로 표시)</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="18" customHeight="1">
-      <c r="A22" s="6" t="inlineStr"/>
-    </row>
-    <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="7" t="inlineStr">
+    <row r="25" ht="18" customHeight="1">
+      <c r="A25" s="6" t="inlineStr"/>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t>● 파일 명명 규칙</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="6" t="inlineStr"/>
-    </row>
-    <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  메인 이미지: folder_name 과 동일 + .png</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">              예) folder_name = 'rw_notarock' → rw_notarock.png</t>
-        </is>
-      </c>
-    </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  갤러리:     2.png 부터 시작 (메인이 1번째이므로)</t>
-        </is>
-      </c>
+      <c r="A27" s="6" t="inlineStr"/>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  상세 본문:  details/ 폴더 안에 1.png 부터 순서대로</t>
+          <t xml:space="preserve">  메인 이미지: folder_name 과 동일 + .png</t>
         </is>
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  사이즈:     size.png (고정 파일명)</t>
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">              예) folder_name = 'rw_notarock' → rw_notarock.png</t>
         </is>
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">  갤러리:     2.png 부터 시작 (메인이 1번째이므로)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="18" customHeight="1">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  상세 본문:  details/ 폴더 안에 1.png 부터 순서대로</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  사이즈:     size.png (고정 파일명)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="18" customHeight="1">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">  영상:       video.mp4 (고정 파일명, mp4 권장)</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="6" t="inlineStr"/>
-    </row>
-    <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="7" t="inlineStr">
-        <is>
-          <t>● 업로드 후 사이트 반영</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="6" t="inlineStr"/>
-    </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  1. 파일을 위 폴더에 저장</t>
-        </is>
-      </c>
+      <c r="A34" s="6" t="inlineStr"/>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  2. GitHub 에 push (또는 RPA 자동)</t>
+      <c r="A35" s="7" t="inlineStr">
+        <is>
+          <t>● 작업 → 사이트 반영 흐름</t>
         </is>
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  3. 1~2분 후 detail_url 에서 확인</t>
-        </is>
-      </c>
+      <c r="A36" s="6" t="inlineStr"/>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="6" t="inlineStr"/>
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1. 위 폴더에 파일 추가/수정</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
-      <c r="A38" s="7" t="inlineStr">
-        <is>
-          <t>● 자주 묻는 질문</t>
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2. npm run dev (또는 npm run build) — sync-images 가 자동 실행되어</t>
         </is>
       </c>
     </row>
     <row r="39" ht="18" customHeight="1">
-      <c r="A39" s="6" t="inlineStr"/>
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     catalog.json 의 image/gallery/details/sizeImage/video 필드가 자동 갱신됩니다</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Q. 폴더 안에 파일을 넣었는데 사이트에 안 보입니다.</t>
+          <t xml:space="preserve">  3. git add . / git commit / git push</t>
         </is>
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  A. 1~2분 정도 빌드/배포 시간 필요. 그래도 안 보이면 파일명 확인 (오타·확장자).</t>
+          <t xml:space="preserve">  4. 1~2분 후 detail_url 에서 확인</t>
         </is>
       </c>
     </row>
@@ -11101,33 +11105,33 @@
       <c r="A42" s="6" t="inlineStr"/>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Q. 갤러리 사진 갯수에 제한이 있나요?</t>
+      <c r="A43" s="7" t="inlineStr">
+        <is>
+          <t>● 자주 묻는 질문</t>
         </is>
       </c>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  A. 제한 없음. 2.png 부터 빈 번호 없이 연속으로 추가.</t>
-        </is>
-      </c>
+      <c r="A44" s="6" t="inlineStr"/>
     </row>
     <row r="45" ht="18" customHeight="1">
-      <c r="A45" s="6" t="inlineStr"/>
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Q. 폴더 안에 파일을 넣었는데 사이트에 안 보입니다.</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Q. 상세 이미지 1번 위에 헤더, 마지막에 푸터 같은 게 있어야 하나요?</t>
+          <t xml:space="preserve">  A. npm run sync-images 실행 후 catalog.json 변경분도 같이 commit 했는지 확인.</t>
         </is>
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  A. 자유. 사이트는 1.png 부터 순서대로만 보여줍니다. 디자인은 자유.</t>
+          <t xml:space="preserve">     1~2분 정도 빌드/배포 시간 필요. 그래도 안 보이면 파일명 확인 (오타·확장자).</t>
         </is>
       </c>
     </row>
@@ -11137,24 +11141,89 @@
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Q. 모든 제품에 영상이나 사이즈 차트가 필요한가요?</t>
+          <t xml:space="preserve">  Q. 갤러리 사진 갯수에 제한이 있나요?</t>
         </is>
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">  A. 제한 없음. 2.png 부터 빈 번호 없이 연속으로 추가.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     중간에 빈 번호 있으면 그 앞까지만 인식됨 (예: 2,3,5 → 2,3 만 사용).</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="18" customHeight="1">
+      <c r="A52" s="6" t="inlineStr"/>
+    </row>
+    <row r="53" ht="18" customHeight="1">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Q. 상세 이미지 1번 위에 헤더, 마지막에 푸터 같은 게 있어야 하나요?</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A. 자유. 사이트는 1.png 부터 순서대로만 보여줍니다. 디자인은 자유.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="18" customHeight="1">
+      <c r="A55" s="6" t="inlineStr"/>
+    </row>
+    <row r="56" ht="18" customHeight="1">
+      <c r="A56" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Q. 모든 제품에 영상이나 사이즈 차트가 필요한가요?</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="18" customHeight="1">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">  A. 아니요. 있으면 표시, 없으면 그 영역 자체가 안 보임. 옵션입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="18" customHeight="1">
+      <c r="A58" s="6" t="inlineStr"/>
+    </row>
+    <row r="59" ht="18" customHeight="1">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Q. npm run sync-images 가 무슨 일을 하나요?</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="18" customHeight="1">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  A. catalog/ 폴더를 스캔해서 각 제품의 image/gallery/details/sizeImage/video</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="18" customHeight="1">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     필드를 catalog.json 에 자동으로 채워줍니다. npm run dev/build 직전 자동 실행.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="6">
-    <mergeCell ref="A38:E38"/>
+    <mergeCell ref="A35:E35"/>
+    <mergeCell ref="A26:E26"/>
+    <mergeCell ref="A43:E43"/>
+    <mergeCell ref="A11:E11"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A23:E23"/>
-    <mergeCell ref="A32:E32"/>
-    <mergeCell ref="A8:E8"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>